<commit_message>
Basic neural network that is working for FYP
1. Manage to make the neural network to work for 25 job instance.
2. Compiled and viewed result from tensorboard and automated test, seems like it works
</commit_message>
<xml_diff>
--- a/(TESTING) automated_testing/automated_test_log.xlsx
+++ b/(TESTING) automated_testing/automated_test_log.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="816" yWindow="3636" windowWidth="17280" windowHeight="9420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="19090" yWindow="-6740" windowWidth="14620" windowHeight="25100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backup" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model tracking" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backup" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$K$1</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -34,13 +35,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="22"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -64,6 +79,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.109375" customWidth="1" min="1" max="1"/>
@@ -1963,6 +1980,744 @@
         <v>9</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-03-31 16:47:00</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>100</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0848</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>6</v>
+      </c>
+      <c r="G39" t="n">
+        <v>25</v>
+      </c>
+      <c r="H39" t="n">
+        <v>50</v>
+      </c>
+      <c r="I39" t="n">
+        <v>60</v>
+      </c>
+      <c r="J39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K39" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-03-31 17:01:03</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.08396000000000001</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
+      <c r="G40" t="n">
+        <v>25</v>
+      </c>
+      <c r="H40" t="n">
+        <v>50</v>
+      </c>
+      <c r="I40" t="n">
+        <v>60</v>
+      </c>
+      <c r="J40" t="n">
+        <v>8</v>
+      </c>
+      <c r="K40" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-03-31 17:28:38</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>S_RPT</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.03792</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" t="n">
+        <v>25</v>
+      </c>
+      <c r="H41" t="n">
+        <v>50</v>
+      </c>
+      <c r="I41" t="n">
+        <v>60</v>
+      </c>
+      <c r="J41" t="n">
+        <v>8</v>
+      </c>
+      <c r="K41" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-03-31 17:52:49</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.08368</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" t="n">
+        <v>25</v>
+      </c>
+      <c r="H42" t="n">
+        <v>50</v>
+      </c>
+      <c r="I42" t="n">
+        <v>60</v>
+      </c>
+      <c r="J42" t="n">
+        <v>8</v>
+      </c>
+      <c r="K42" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-03-31 22:45:19</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>100</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>6</v>
+      </c>
+      <c r="G43" t="n">
+        <v>25</v>
+      </c>
+      <c r="H43" t="n">
+        <v>50</v>
+      </c>
+      <c r="I43" t="n">
+        <v>60</v>
+      </c>
+      <c r="J43" t="n">
+        <v>8</v>
+      </c>
+      <c r="K43" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-04-02 18:44:21</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.08124000000000001</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>6</v>
+      </c>
+      <c r="G44" t="n">
+        <v>25</v>
+      </c>
+      <c r="H44" t="n">
+        <v>50</v>
+      </c>
+      <c r="I44" t="n">
+        <v>60</v>
+      </c>
+      <c r="J44" t="n">
+        <v>8</v>
+      </c>
+      <c r="K44" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-04-03 04:38:26</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.08172</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>6</v>
+      </c>
+      <c r="G45" t="n">
+        <v>25</v>
+      </c>
+      <c r="H45" t="n">
+        <v>50</v>
+      </c>
+      <c r="I45" t="n">
+        <v>60</v>
+      </c>
+      <c r="J45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-04-03 04:39:51</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>FIFO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.09616</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>6</v>
+      </c>
+      <c r="G46" t="n">
+        <v>25</v>
+      </c>
+      <c r="H46" t="n">
+        <v>50</v>
+      </c>
+      <c r="I46" t="n">
+        <v>60</v>
+      </c>
+      <c r="J46" t="n">
+        <v>8</v>
+      </c>
+      <c r="K46" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-04-03 04:41:23</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>S_RPT</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.03368</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>6</v>
+      </c>
+      <c r="G47" t="n">
+        <v>25</v>
+      </c>
+      <c r="H47" t="n">
+        <v>50</v>
+      </c>
+      <c r="I47" t="n">
+        <v>60</v>
+      </c>
+      <c r="J47" t="n">
+        <v>8</v>
+      </c>
+      <c r="K47" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-04-03 04:42:50</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>MTWR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.06844</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>6</v>
+      </c>
+      <c r="G48" t="n">
+        <v>25</v>
+      </c>
+      <c r="H48" t="n">
+        <v>50</v>
+      </c>
+      <c r="I48" t="n">
+        <v>60</v>
+      </c>
+      <c r="J48" t="n">
+        <v>8</v>
+      </c>
+      <c r="K48" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-04-03 04:57:19</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.08416</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>6</v>
+      </c>
+      <c r="G49" t="n">
+        <v>25</v>
+      </c>
+      <c r="H49" t="n">
+        <v>50</v>
+      </c>
+      <c r="I49" t="n">
+        <v>60</v>
+      </c>
+      <c r="J49" t="n">
+        <v>8</v>
+      </c>
+      <c r="K49" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:01:17</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>FIFO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.09498666666666666</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>6</v>
+      </c>
+      <c r="G50" t="n">
+        <v>25</v>
+      </c>
+      <c r="H50" t="n">
+        <v>50</v>
+      </c>
+      <c r="I50" t="n">
+        <v>60</v>
+      </c>
+      <c r="J50" t="n">
+        <v>8</v>
+      </c>
+      <c r="K50" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:05:35</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>S_RPT</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.03908</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>6</v>
+      </c>
+      <c r="G51" t="n">
+        <v>25</v>
+      </c>
+      <c r="H51" t="n">
+        <v>50</v>
+      </c>
+      <c r="I51" t="n">
+        <v>60</v>
+      </c>
+      <c r="J51" t="n">
+        <v>8</v>
+      </c>
+      <c r="K51" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:09:35</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MTWR</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>0.06785333333333333</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" t="n">
+        <v>25</v>
+      </c>
+      <c r="H52" t="n">
+        <v>50</v>
+      </c>
+      <c r="I52" t="n">
+        <v>60</v>
+      </c>
+      <c r="J52" t="n">
+        <v>8</v>
+      </c>
+      <c r="K52" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:32:17</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0.082704</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>6</v>
+      </c>
+      <c r="G53" t="n">
+        <v>25</v>
+      </c>
+      <c r="H53" t="n">
+        <v>50</v>
+      </c>
+      <c r="I53" t="n">
+        <v>60</v>
+      </c>
+      <c r="J53" t="n">
+        <v>8</v>
+      </c>
+      <c r="K53" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:38:44</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>FIFO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0.096792</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>6</v>
+      </c>
+      <c r="G54" t="n">
+        <v>25</v>
+      </c>
+      <c r="H54" t="n">
+        <v>50</v>
+      </c>
+      <c r="I54" t="n">
+        <v>60</v>
+      </c>
+      <c r="J54" t="n">
+        <v>8</v>
+      </c>
+      <c r="K54" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:45:46</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>S_RPT</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.038784</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>6</v>
+      </c>
+      <c r="G55" t="n">
+        <v>25</v>
+      </c>
+      <c r="H55" t="n">
+        <v>50</v>
+      </c>
+      <c r="I55" t="n">
+        <v>60</v>
+      </c>
+      <c r="J55" t="n">
+        <v>8</v>
+      </c>
+      <c r="K55" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2025-04-03 05:52:20</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>MTWR</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0.06765599999999999</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>[10, 12]</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>6</v>
+      </c>
+      <c r="G56" t="n">
+        <v>25</v>
+      </c>
+      <c r="H56" t="n">
+        <v>50</v>
+      </c>
+      <c r="I56" t="n">
+        <v>60</v>
+      </c>
+      <c r="J56" t="n">
+        <v>8</v>
+      </c>
+      <c r="K56" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1">
     <sortState ref="A2:K27">
@@ -1974,6 +2729,77 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="54.109375" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="28.8" customHeight="1">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tuning changes made </t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A2C_v2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Added reward function for scheduling without delay </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>A2C_v3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Agent still take illegal actions, but able to complete the episode</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Increased reward for manage to schedule to  +5 and applied tanh squashing for the reward from self.allowance with a hardcoded scaling factor of 1000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>